<commit_message>
Update Feefo and Review reports for 2026-09-07T02:48:03Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -487,7 +487,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1142809</t>
+          <t>1018553</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -499,14 +499,14 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1142809&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1018553&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1281098</t>
+          <t>1091204</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -518,33 +518,33 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1281098&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1091204&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1308378</t>
+          <t>1158524</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1308378&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1158524&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1341083</t>
+          <t>1208903</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -556,14 +556,14 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1341083&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1208903&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1420726</t>
+          <t>1249874</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -575,33 +575,33 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1420726&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1249874&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1436341</t>
+          <t>1307741</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1436341&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1307741&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1458521</t>
+          <t>1347156</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -613,14 +613,14 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1458521&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1347156&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1478705</t>
+          <t>1347160</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -632,14 +632,14 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1478705&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1347160&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1624715</t>
+          <t>1362744</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -651,14 +651,14 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1624715&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1362744&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>255970</t>
+          <t>1389021</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -670,33 +670,33 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=255970&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1389021&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>545355</t>
+          <t>1476097</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=545355&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1476097&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>550715</t>
+          <t>1498343</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -708,14 +708,14 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=550715&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1498343&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>868202</t>
+          <t>1526108</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -727,14 +727,14 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=868202&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1526108&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>920040</t>
+          <t>1544515</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -746,26 +746,311 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=920040&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1544515&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>999592</t>
+          <t>1546075</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=999592&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1546075&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>1546290</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="n">
+        <v>3</v>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1546290&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>1574068</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="n">
+        <v>2</v>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1574068&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>1602499</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="n">
+        <v>2</v>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1602499&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>1603180</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="n">
+        <v>2</v>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1603180&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>1609160</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1609160&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>469358</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="n">
+        <v>3</v>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>499153</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="n">
+        <v>2</v>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=499153&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>601537</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="n">
+        <v>2</v>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=601537&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>701046</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="n">
+        <v>4</v>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=701046&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>718063</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="n">
+        <v>2</v>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=718063&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>764151</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="n">
+        <v>3</v>
+      </c>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=764151&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>806693</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="n">
+        <v>2</v>
+      </c>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=806693&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>860988</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="n">
+        <v>2</v>
+      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=860988&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>937471</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="n">
+        <v>2</v>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=937471&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>960160</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="n">
+        <v>2</v>
+      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=960160&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Feefo and Review reports for 2026-09-14T03:16:08Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,26 +468,26 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1008277</t>
+          <t>1062346</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1008277&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1062346&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1018553</t>
+          <t>1170247</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -499,14 +499,14 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1018553&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1170247&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1091204</t>
+          <t>1234302</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -518,14 +518,14 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1091204&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1234302&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1158524</t>
+          <t>1431678</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -537,14 +537,14 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1158524&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1431678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1208903</t>
+          <t>1486879</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -556,14 +556,14 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1208903&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1486879&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1249874</t>
+          <t>1500483</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -575,33 +575,33 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1249874&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1500483&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1307741</t>
+          <t>1508805</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1307741&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1508805&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1347156</t>
+          <t>1532914</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -613,14 +613,14 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1347156&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1532914&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1347160</t>
+          <t>1600852</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -632,33 +632,33 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1347160&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1600852&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1362744</t>
+          <t>1602499</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1362744&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1602499&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1389021</t>
+          <t>1616105</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -670,33 +670,33 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1389021&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1616105&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1476097</t>
+          <t>469358</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1476097&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1498343</t>
+          <t>684433</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -708,14 +708,14 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1498343&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=684433&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1526108</t>
+          <t>764151</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -727,14 +727,14 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1526108&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=764151&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1544515</t>
+          <t>930897</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -746,311 +746,26 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1544515&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=930897&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1546075</t>
+          <t>991741</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1546075&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>1546290</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="n">
-        <v>3</v>
-      </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1546290&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>1574068</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="n">
-        <v>2</v>
-      </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1574068&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>1602499</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="n">
-        <v>2</v>
-      </c>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1602499&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>1603180</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="n">
-        <v>2</v>
-      </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1603180&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>1609160</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="n">
-        <v>2</v>
-      </c>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1609160&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>469358</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="n">
-        <v>3</v>
-      </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>499153</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="n">
-        <v>2</v>
-      </c>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=499153&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>601537</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="n">
-        <v>2</v>
-      </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=601537&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>701046</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="n">
-        <v>4</v>
-      </c>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=701046&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>718063</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="n">
-        <v>2</v>
-      </c>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=718063&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>764151</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="n">
-        <v>3</v>
-      </c>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=764151&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>806693</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr"/>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="n">
-        <v>2</v>
-      </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=806693&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>860988</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="n">
-        <v>2</v>
-      </c>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=860988&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>937471</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="n">
-        <v>2</v>
-      </c>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=937471&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>960160</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr"/>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="n">
-        <v>2</v>
-      </c>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=960160&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=991741&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Feefo and Review reports for 2026-09-21T03:13:43Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,26 +468,26 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1062346</t>
+          <t>1071561</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1062346&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1071561&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1170247</t>
+          <t>1080185</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -499,14 +499,14 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1170247&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1080185&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1234302</t>
+          <t>1223789</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -518,14 +518,14 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1234302&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1223789&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1431678</t>
+          <t>1260374</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -537,14 +537,14 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1431678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1260374&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1486879</t>
+          <t>1416431</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -556,14 +556,14 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1486879&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1416431&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1500483</t>
+          <t>1531914</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -575,14 +575,14 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1500483&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1531914&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1508805</t>
+          <t>1532597</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -594,14 +594,14 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1508805&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1532597&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1532914</t>
+          <t>1578263</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -613,14 +613,14 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1532914&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1578263&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1600852</t>
+          <t>1587950</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -632,33 +632,33 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1600852&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1587950&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1602499</t>
+          <t>1606886</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1602499&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1606886&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1616105</t>
+          <t>236583</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -670,14 +670,14 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1616105&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=236583&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>469358</t>
+          <t>250985</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -689,14 +689,14 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=250985&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>684433</t>
+          <t>469358</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -708,14 +708,14 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=684433&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>764151</t>
+          <t>501250</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -727,14 +727,14 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=764151&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=501250&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>930897</t>
+          <t>684433</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -746,14 +746,14 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=930897&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=684433&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>991741</t>
+          <t>764151</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -765,7 +765,121 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=991741&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=764151&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>769547</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="n">
+        <v>2</v>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=769547&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>770314</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="n">
+        <v>2</v>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=770314&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>844846</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="n">
+        <v>2</v>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=844846&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>963962</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="n">
+        <v>2</v>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=963962&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>991876</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=991876&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>999592</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="n">
+        <v>2</v>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=999592&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Feefo and Review reports for 2026-09-28T03:32:19Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1071561</t>
+          <t>1018553</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -480,14 +480,14 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1071561&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1018553&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1080185</t>
+          <t>1025564</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -499,14 +499,14 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1080185&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1025564&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1223789</t>
+          <t>1030998</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -518,14 +518,14 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1223789&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1030998&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1260374</t>
+          <t>1039106</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -537,33 +537,33 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1260374&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1039106&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1416431</t>
+          <t>1049381</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1416431&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1049381&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1531914</t>
+          <t>1184400</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -575,14 +575,14 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1531914&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1184400&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1532597</t>
+          <t>1322572</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -594,14 +594,14 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1532597&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1322572&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1578263</t>
+          <t>1399988</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -613,14 +613,14 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1578263&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1399988&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1587950</t>
+          <t>1431678</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -632,14 +632,14 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1587950&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1431678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1606886</t>
+          <t>1487346</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -651,14 +651,14 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1606886&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1487346&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>236583</t>
+          <t>1488964</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -670,33 +670,33 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=236583&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1488964&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>250985</t>
+          <t>1500483</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=250985&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1500483&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>469358</t>
+          <t>1529758</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -708,14 +708,14 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1529758&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>501250</t>
+          <t>1539551</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -727,14 +727,14 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=501250&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1539551&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>684433</t>
+          <t>1544832</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -746,14 +746,14 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=684433&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1544832&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>764151</t>
+          <t>1548271</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -765,33 +765,33 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=764151&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1548271&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>769547</t>
+          <t>1578263</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=769547&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1578263&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>770314</t>
+          <t>1586736</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -803,52 +803,52 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=770314&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1586736&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>844846</t>
+          <t>1602499</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=844846&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1602499&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>963962</t>
+          <t>1602612</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=963962&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1602612&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>991876</t>
+          <t>1603180</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
@@ -860,14 +860,14 @@
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=991876&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1603180&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>999592</t>
+          <t>380247</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
@@ -879,7 +879,197 @@
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=999592&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=380247&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>545355</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="n">
+        <v>2</v>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=545355&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>631219</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="n">
+        <v>2</v>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=631219&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>764151</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="n">
+        <v>3</v>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=764151&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>799432</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="n">
+        <v>2</v>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=799432&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>802144</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="n">
+        <v>2</v>
+      </c>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=802144&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>818651</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="n">
+        <v>2</v>
+      </c>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=818651&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>908949</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="n">
+        <v>2</v>
+      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=908949&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>930897</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="n">
+        <v>2</v>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=930897&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>960222</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="n">
+        <v>2</v>
+      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=960222&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>991747</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="n">
+        <v>2</v>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=991747&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Feefo and Review reports for 2026-10-05T03:59:00Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,26 +468,26 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1018553</t>
+          <t>100458</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1018553&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=100458&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1025564</t>
+          <t>1127852</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -499,14 +499,14 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1025564&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1127852&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1030998</t>
+          <t>1142238</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -518,14 +518,14 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1030998&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1142238&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1039106</t>
+          <t>1244120</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -537,14 +537,14 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1039106&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1244120&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1049381</t>
+          <t>1324828</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -556,14 +556,14 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1049381&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1324828&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1184400</t>
+          <t>1328533</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -575,14 +575,14 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1184400&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1328533&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1322572</t>
+          <t>1343257</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -594,14 +594,14 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1322572&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1343257&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1399988</t>
+          <t>1347156</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -613,14 +613,14 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1399988&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1347156&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1431678</t>
+          <t>1347160</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -632,14 +632,14 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1431678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1347160&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1487346</t>
+          <t>141541</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -651,14 +651,14 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1487346&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=141541&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1488964</t>
+          <t>1460477</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -670,33 +670,33 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1488964&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1460477&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1500483</t>
+          <t>1491899</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1500483&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1491899&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1529758</t>
+          <t>1505632</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -708,14 +708,14 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1529758&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1505632&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1539551</t>
+          <t>1505664</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -727,14 +727,14 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1539551&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1505664&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1544832</t>
+          <t>1527760</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -746,14 +746,14 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1544832&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1527760&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1548271</t>
+          <t>1540360</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -765,33 +765,33 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1548271&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1540360&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1578263</t>
+          <t>1544832</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1578263&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1544832&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1586736</t>
+          <t>1560549</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -803,52 +803,52 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1586736&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1560549&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1602499</t>
+          <t>1580286</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1602499&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1580286&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1602612</t>
+          <t>1586903</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1602612&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1586903&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1603180</t>
+          <t>1602499</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
@@ -860,33 +860,33 @@
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1603180&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1602499&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>380247</t>
+          <t>1602612</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=380247&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1602612&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>545355</t>
+          <t>1617713</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
@@ -898,14 +898,14 @@
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=545355&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1617713&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>631219</t>
+          <t>250985</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
@@ -917,33 +917,33 @@
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=631219&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=250985&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>764151</t>
+          <t>307261</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=764151&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=307261&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>799432</t>
+          <t>469358</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
@@ -955,14 +955,14 @@
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=799432&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>802144</t>
+          <t>499724</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
@@ -974,14 +974,14 @@
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=802144&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=499724&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>818651</t>
+          <t>510573</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
@@ -993,14 +993,14 @@
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=818651&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=510573&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>908949</t>
+          <t>752970</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
@@ -1012,14 +1012,14 @@
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=908949&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=752970&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>930897</t>
+          <t>764151</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
@@ -1031,14 +1031,14 @@
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=930897&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=764151&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>960222</t>
+          <t>824963</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
@@ -1050,14 +1050,14 @@
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=960222&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=824963&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>991747</t>
+          <t>903222</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
@@ -1069,7 +1069,26 @@
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=991747&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=903222&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>944166</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr"/>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="n">
+        <v>2</v>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=944166&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Feefo and Review reports for 2026-10-12T04:14:48Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,26 +468,26 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>100458</t>
+          <t>1149991</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=100458&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1149991&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1127852</t>
+          <t>1189991</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -499,33 +499,33 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1127852&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1189991&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1142238</t>
+          <t>1239838</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1142238&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1239838&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1244120</t>
+          <t>1286676</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -537,33 +537,33 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1244120&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1286676&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1324828</t>
+          <t>1308378</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1324828&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1308378&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1328533</t>
+          <t>1332189</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -575,33 +575,33 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1328533&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1332189&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1343257</t>
+          <t>1334332</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1343257&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1334332&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1347156</t>
+          <t>1344943</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -613,14 +613,14 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1347156&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1344943&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1347160</t>
+          <t>1359483</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -632,14 +632,14 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1347160&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1359483&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>141541</t>
+          <t>1362511</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -651,14 +651,14 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=141541&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1362511&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1460477</t>
+          <t>1398352</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -670,33 +670,33 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1460477&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1398352&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1491899</t>
+          <t>1406717</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1491899&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1406717&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1505632</t>
+          <t>1452883</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -708,14 +708,14 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1505632&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1452883&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1505664</t>
+          <t>1491899</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -727,14 +727,14 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1505664&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1491899&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1527760</t>
+          <t>1497676</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -746,14 +746,14 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1527760&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1497676&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1540360</t>
+          <t>1500483</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -765,14 +765,14 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1540360&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1500483&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1544832</t>
+          <t>1506831</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
@@ -784,14 +784,14 @@
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1544832&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1506831&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1560549</t>
+          <t>1531914</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -803,14 +803,14 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1560549&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1531914&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1580286</t>
+          <t>1539679</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
@@ -822,14 +822,14 @@
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1580286&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1539679&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1586903</t>
+          <t>1541669</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
@@ -841,14 +841,14 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1586903&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1541669&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1602499</t>
+          <t>1560710</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
@@ -860,33 +860,33 @@
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1602499&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1560710&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1602612</t>
+          <t>1578393</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1602612&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1578393&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1617713</t>
+          <t>159976</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
@@ -898,33 +898,33 @@
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1617713&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=159976&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>250985</t>
+          <t>1602499</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=250985&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1602499&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>307261</t>
+          <t>1602612</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
@@ -936,14 +936,14 @@
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=307261&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1602612&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>469358</t>
+          <t>307533</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
@@ -955,14 +955,14 @@
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=307533&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>499724</t>
+          <t>460660</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
@@ -974,33 +974,33 @@
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=499724&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=460660&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>510573</t>
+          <t>469358</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=510573&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>752970</t>
+          <t>545355</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
@@ -1012,14 +1012,14 @@
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=752970&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=545355&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>764151</t>
+          <t>621809</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
@@ -1031,14 +1031,14 @@
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=764151&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=621809&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>824963</t>
+          <t>684433</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
@@ -1050,33 +1050,33 @@
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=824963&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=684433&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>903222</t>
+          <t>804990</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=903222&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=804990&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>944166</t>
+          <t>841587</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
@@ -1088,7 +1088,45 @@
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=944166&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=841587&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>915292</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr"/>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="n">
+        <v>2</v>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=915292&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>991747</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr"/>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="n">
+        <v>3</v>
+      </c>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=991747&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Feefo and Review reports for 2026-10-19T03:11:48Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1149991</t>
+          <t>1016235</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -480,14 +480,14 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1149991&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1016235&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1189991</t>
+          <t>1047034</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -499,33 +499,33 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1189991&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1047034&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1239838</t>
+          <t>1170247</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1239838&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1170247&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1286676</t>
+          <t>1180998</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -537,14 +537,14 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1286676&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1180998&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1308378</t>
+          <t>1313480</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -556,14 +556,14 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1308378&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1313480&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1332189</t>
+          <t>1341083</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -575,33 +575,33 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1332189&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1341083&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1334332</t>
+          <t>1347156</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1334332&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1347156&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1344943</t>
+          <t>1359483</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -613,14 +613,14 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1344943&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1359483&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1359483</t>
+          <t>1361615</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -632,14 +632,14 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1359483&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1361615&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1362511</t>
+          <t>1371380</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -651,33 +651,33 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1362511&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1371380&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1398352</t>
+          <t>1372929</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1398352&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1372929&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1406717</t>
+          <t>1381077</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -689,14 +689,14 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1406717&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1381077&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1452883</t>
+          <t>1435842</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -708,14 +708,14 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1452883&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1435842&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1491899</t>
+          <t>1466482</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -727,14 +727,14 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1491899&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1466482&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1497676</t>
+          <t>1470605</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -746,14 +746,14 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1497676&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1470605&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1500483</t>
+          <t>1476097</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -765,14 +765,14 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1500483&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1476097&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1506831</t>
+          <t>1480636</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
@@ -784,14 +784,14 @@
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1506831&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1480636&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1531914</t>
+          <t>1487003</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -803,14 +803,14 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1531914&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1487003&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1539679</t>
+          <t>1488674</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
@@ -822,14 +822,14 @@
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1539679&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1488674&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1541669</t>
+          <t>1500474</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
@@ -841,14 +841,14 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1541669&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1500474&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1560710</t>
+          <t>1503127</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
@@ -860,14 +860,14 @@
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1560710&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1503127&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1578393</t>
+          <t>1505664</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
@@ -879,14 +879,14 @@
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1578393&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1505664&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>159976</t>
+          <t>1578393</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
@@ -898,14 +898,14 @@
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=159976&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1578393&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>1602499</t>
+          <t>1589504</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
@@ -917,52 +917,52 @@
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1602499&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1589504&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1602612</t>
+          <t>1602499</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1602612&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1602499&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>307533</t>
+          <t>1603180</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=307533&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1603180&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>460660</t>
+          <t>255970</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
@@ -974,33 +974,33 @@
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=460660&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=255970&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>469358</t>
+          <t>330009</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=330009&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>545355</t>
+          <t>348268</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
@@ -1012,33 +1012,33 @@
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=545355&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=348268&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>621809</t>
+          <t>469358</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=621809&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>684433</t>
+          <t>512339</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
@@ -1050,33 +1050,33 @@
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=684433&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=512339&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>804990</t>
+          <t>614510</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=804990&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=614510&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>841587</t>
+          <t>663976</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
@@ -1088,14 +1088,14 @@
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=841587&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=663976&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>915292</t>
+          <t>684433</t>
         </is>
       </c>
       <c r="B35" t="inlineStr"/>
@@ -1107,24 +1107,138 @@
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=915292&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=684433&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>991747</t>
+          <t>730583</t>
         </is>
       </c>
       <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=730583&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>764151</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr"/>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="n">
+        <v>2</v>
+      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=764151&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>786481</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr"/>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="n">
+        <v>2</v>
+      </c>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=786481&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>893398</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr"/>
+      <c r="C39" t="inlineStr"/>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="n">
+        <v>2</v>
+      </c>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=893398&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>963254</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr"/>
+      <c r="C40" t="inlineStr"/>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="n">
+        <v>3</v>
+      </c>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=963254&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>986868</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr"/>
+      <c r="C41" t="inlineStr"/>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="n">
+        <v>3</v>
+      </c>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=986868&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>991747</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr"/>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="n">
+        <v>2</v>
+      </c>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr">
         <is>
           <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=991747&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>

</xml_diff>

<commit_message>
Update Feefo and Review reports for 2026-10-26T03:08:45Z
</commit_message>
<xml_diff>
--- a/data/recent_reviews_web_ready.xlsx
+++ b/data/recent_reviews_web_ready.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,7 +468,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1016235</t>
+          <t>1003991</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -480,14 +480,14 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1016235&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1003991&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1047034</t>
+          <t>1061678</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -499,14 +499,14 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1047034&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1061678&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1170247</t>
+          <t>1102114</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -518,14 +518,14 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1170247&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1102114&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1180998</t>
+          <t>1130264</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -537,14 +537,14 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1180998&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1130264&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1313480</t>
+          <t>1130272</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -556,14 +556,14 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1313480&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1130272&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1341083</t>
+          <t>1249874</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -575,14 +575,14 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1341083&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1249874&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1347156</t>
+          <t>1299630</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -594,14 +594,14 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1347156&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1299630&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1359483</t>
+          <t>1351207</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -613,14 +613,14 @@
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1359483&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1351207&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1361615</t>
+          <t>1387886</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -632,14 +632,14 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1361615&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1387886&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1371380</t>
+          <t>1473165</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -651,33 +651,33 @@
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1371380&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1473165&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1372929</t>
+          <t>1480130</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1372929&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1480130&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1381077</t>
+          <t>1481587</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -689,14 +689,14 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1381077&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1481587&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1435842</t>
+          <t>1486089</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -708,14 +708,14 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1435842&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1486089&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1466482</t>
+          <t>1491248</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -727,14 +727,14 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1466482&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1491248&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1470605</t>
+          <t>1503123</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -746,14 +746,14 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1470605&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1503123&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1476097</t>
+          <t>1506034</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -765,14 +765,14 @@
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1476097&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1506034&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1480636</t>
+          <t>1527319</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
@@ -784,14 +784,14 @@
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1480636&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1527319&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1487003</t>
+          <t>1540005</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -803,14 +803,14 @@
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1487003&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1540005&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1488674</t>
+          <t>1547383</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
@@ -822,14 +822,14 @@
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1488674&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1547383&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1500474</t>
+          <t>1553919</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
@@ -841,14 +841,14 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1500474&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1553919&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1503127</t>
+          <t>1553937</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
@@ -860,14 +860,14 @@
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1503127&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1553937&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1505664</t>
+          <t>1601601</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
@@ -879,90 +879,90 @@
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1505664&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1601601&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1578393</t>
+          <t>1602499</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1578393&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1602499&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>1589504</t>
+          <t>1603192</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1589504&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1603192&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1602499</t>
+          <t>1608977</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1602499&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1608977&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>1603180</t>
+          <t>1618152</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1603180&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1618152&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>255970</t>
+          <t>1624707</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
@@ -974,14 +974,14 @@
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=255970&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1624707&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>330009</t>
+          <t>1627286</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
@@ -993,14 +993,14 @@
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=330009&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1627286&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>348268</t>
+          <t>1633927</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
@@ -1012,52 +1012,52 @@
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=348268&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1633927&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>469358</t>
+          <t>1635135</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=1635135&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>512339</t>
+          <t>352545</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=512339&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=352545&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>614510</t>
+          <t>469358</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
@@ -1069,14 +1069,14 @@
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=614510&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=469358&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>663976</t>
+          <t>501293</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
@@ -1088,14 +1088,14 @@
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=663976&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=501293&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>684433</t>
+          <t>512339</t>
         </is>
       </c>
       <c r="B35" t="inlineStr"/>
@@ -1107,14 +1107,14 @@
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=684433&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=512339&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>730583</t>
+          <t>545355</t>
         </is>
       </c>
       <c r="B36" t="inlineStr"/>
@@ -1126,14 +1126,14 @@
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=730583&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=545355&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>764151</t>
+          <t>566001</t>
         </is>
       </c>
       <c r="B37" t="inlineStr"/>
@@ -1145,33 +1145,33 @@
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=764151&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=566001&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>786481</t>
+          <t>566057</t>
         </is>
       </c>
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=786481&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=566057&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>893398</t>
+          <t>607975</t>
         </is>
       </c>
       <c r="B39" t="inlineStr"/>
@@ -1183,33 +1183,33 @@
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=893398&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=607975&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>963254</t>
+          <t>752970</t>
         </is>
       </c>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=963254&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=752970&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>986868</t>
+          <t>764151</t>
         </is>
       </c>
       <c r="B41" t="inlineStr"/>
@@ -1221,26 +1221,159 @@
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=986868&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=764151&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>991747</t>
+          <t>786481</t>
         </is>
       </c>
       <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr"/>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
-          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=991747&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=786481&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>799255</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr"/>
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="n">
+        <v>2</v>
+      </c>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=799255&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>841587</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr"/>
+      <c r="C44" t="inlineStr"/>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="n">
+        <v>2</v>
+      </c>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=841587&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>857670</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr"/>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="n">
+        <v>2</v>
+      </c>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=857670&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>944166</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr"/>
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="n">
+        <v>3</v>
+      </c>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=944166&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>963254</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr"/>
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="n">
+        <v>2</v>
+      </c>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=963254&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>971143</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr"/>
+      <c r="C48" t="inlineStr"/>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="n">
+        <v>2</v>
+      </c>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=971143&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>991741</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr"/>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="n">
+        <v>2</v>
+      </c>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>https://www.feefo.com/en-US/reviews/notonthehighstreet-com/products/*?sku=991741&amp;displayFeedbackType=PRODUCT&amp;timeFrame=ALL</t>
         </is>
       </c>
     </row>

</xml_diff>